<commit_message>
Weekly availability list refresh
</commit_message>
<xml_diff>
--- a/files/availability-list-october-2026.xlsx
+++ b/files/availability-list-october-2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I958"/>
+  <dimension ref="A1:I963"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34698,12 +34698,12 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>15653</t>
+          <t>16492</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>SORBUS 'Eastern Promise'</t>
+          <t>SORBUS  'Golden Wonder'</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
@@ -34713,34 +34713,38 @@
       </c>
       <c r="D879" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>B/ R</t>
         </is>
       </c>
       <c r="E879" t="inlineStr">
         <is>
-          <t>150-200cm</t>
-        </is>
-      </c>
-      <c r="F879" t="inlineStr"/>
+          <t>400-450cm</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>14/16</t>
+        </is>
+      </c>
       <c r="G879" t="inlineStr">
         <is>
-          <t>£45.00</t>
+          <t>£180.00</t>
         </is>
       </c>
       <c r="H879" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I879" s="4" t="inlineStr"/>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>16495</t>
+          <t>16491</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>SORBUS 'Eastern Promise'</t>
+          <t>SORBUS  'Golden Wonder'</t>
         </is>
       </c>
       <c r="C880" t="inlineStr">
@@ -34750,33 +34754,33 @@
       </c>
       <c r="D880" t="inlineStr">
         <is>
-          <t>25Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>300-350cm</t>
+          <t>350-400cm</t>
         </is>
       </c>
       <c r="F880" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>12/14</t>
         </is>
       </c>
       <c r="G880" t="inlineStr">
         <is>
-          <t>£145.00</t>
+          <t>£155.00</t>
         </is>
       </c>
       <c r="H880" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I880" s="4" t="inlineStr"/>
     </row>
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>17681</t>
+          <t>15653</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
@@ -34791,107 +34795,111 @@
       </c>
       <c r="D881" t="inlineStr">
         <is>
-          <t>B/R</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>300-350 cm</t>
-        </is>
-      </c>
-      <c r="F881" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>150-200cm</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr"/>
       <c r="G881" t="inlineStr">
         <is>
-          <t>£105.00</t>
+          <t>£45.00</t>
         </is>
       </c>
       <c r="H881" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I881" s="4" t="inlineStr"/>
     </row>
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>17216</t>
+          <t>16495</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>SORBUS 'Olympic Flame'</t>
+          <t>SORBUS 'Eastern Promise'</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Mountain Ash</t>
         </is>
       </c>
       <c r="D882" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>25Ltr</t>
         </is>
       </c>
       <c r="E882" t="inlineStr">
         <is>
-          <t>100-125cm</t>
-        </is>
-      </c>
-      <c r="F882" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G882" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£145.00</t>
         </is>
       </c>
       <c r="H882" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="I882" s="4" t="inlineStr"/>
     </row>
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>15741</t>
+          <t>17681</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>SORBUS 'Olympic Flame'</t>
+          <t>SORBUS 'Eastern Promise'</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Mountain Ash</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>175 -200cm</t>
-        </is>
-      </c>
-      <c r="F883" t="inlineStr"/>
+          <t>300-350 cm</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G883" t="inlineStr">
         <is>
-          <t>£55.00</t>
+          <t>£105.00</t>
         </is>
       </c>
       <c r="H883" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I883" s="4" t="inlineStr"/>
     </row>
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>17680</t>
+          <t>17216</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
@@ -34906,33 +34914,29 @@
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>B/ R</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E884" t="inlineStr">
         <is>
-          <t>350-400cm</t>
-        </is>
-      </c>
-      <c r="F884" t="inlineStr">
-        <is>
-          <t>12/14</t>
-        </is>
-      </c>
+          <t>100-125cm</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr"/>
       <c r="G884" t="inlineStr">
         <is>
-          <t>£155.00</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H884" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="I884" s="4" t="inlineStr"/>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>17679</t>
+          <t>15741</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
@@ -34947,96 +34951,100 @@
       </c>
       <c r="D885" t="inlineStr">
         <is>
-          <t>B/R</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>300-350cm</t>
-        </is>
-      </c>
-      <c r="F885" t="inlineStr">
-        <is>
-          <t>10/12</t>
-        </is>
-      </c>
+          <t>175 -200cm</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr"/>
       <c r="G885" t="inlineStr">
         <is>
-          <t>£130.00</t>
+          <t>£55.00</t>
         </is>
       </c>
       <c r="H885" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I885" s="4" t="inlineStr"/>
     </row>
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>13272</t>
+          <t>17680</t>
         </is>
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>SORBUS aria 'Lutescens'</t>
+          <t>SORBUS 'Olympic Flame'</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>Whitebeam</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="D886" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>B/ R</t>
         </is>
       </c>
       <c r="E886" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F886" t="inlineStr"/>
+          <t>350-400cm</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>12/14</t>
+        </is>
+      </c>
       <c r="G886" t="inlineStr">
         <is>
-          <t>£31.50</t>
+          <t>£155.00</t>
         </is>
       </c>
       <c r="H886" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I886" s="4" t="inlineStr"/>
     </row>
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>13273</t>
+          <t>17679</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>SORBUS aria 'Magnifica'</t>
+          <t>SORBUS 'Olympic Flame'</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>Whitebeam</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
         <is>
-          <t>150-200cm</t>
-        </is>
-      </c>
-      <c r="F887" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G887" t="inlineStr">
         <is>
-          <t>£34.50</t>
+          <t>£130.00</t>
         </is>
       </c>
       <c r="H887" t="n">
@@ -35047,12 +35055,12 @@
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>16489</t>
+          <t>13272</t>
         </is>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>SORBUS aria 'Magnifica'</t>
+          <t>SORBUS aria 'Lutescens'</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
@@ -35062,148 +35070,148 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>300-350cm</t>
-        </is>
-      </c>
-      <c r="F888" t="inlineStr">
-        <is>
-          <t>10/12</t>
-        </is>
-      </c>
+          <t>90-120cm</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr"/>
       <c r="G888" t="inlineStr">
         <is>
-          <t>£175.00</t>
+          <t>£31.50</t>
         </is>
       </c>
       <c r="H888" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I888" s="4" t="inlineStr"/>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t>17395</t>
+          <t>13273</t>
         </is>
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia</t>
+          <t>SORBUS aria 'Magnifica'</t>
         </is>
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>Rowan or Mountain Ash</t>
+          <t>Whitebeam</t>
         </is>
       </c>
       <c r="D889" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E889" t="inlineStr">
         <is>
-          <t>120-150cm</t>
+          <t>150-200cm</t>
         </is>
       </c>
       <c r="F889" t="inlineStr"/>
       <c r="G889" t="inlineStr">
         <is>
-          <t>£24.00</t>
+          <t>£34.50</t>
         </is>
       </c>
       <c r="H889" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I889" s="4" t="inlineStr"/>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
         <is>
-          <t>15652</t>
+          <t>16489</t>
         </is>
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia</t>
+          <t>SORBUS aria 'Magnifica'</t>
         </is>
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>Rowan or Mountain Ash</t>
+          <t>Whitebeam</t>
         </is>
       </c>
       <c r="D890" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E890" t="inlineStr">
         <is>
-          <t>200-250cm</t>
-        </is>
-      </c>
-      <c r="F890" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G890" t="inlineStr">
         <is>
-          <t>£48.00</t>
+          <t>£175.00</t>
         </is>
       </c>
       <c r="H890" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I890" s="4" t="inlineStr"/>
     </row>
     <row r="891">
       <c r="A891" t="inlineStr">
         <is>
-          <t>17039</t>
+          <t>16490</t>
         </is>
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia</t>
+          <t>SORBUS aria 'Magnifica'</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>Rowan or Mountain Ash</t>
+          <t>Whitebeam</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>35 Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E891" t="inlineStr">
         <is>
-          <t>350-400 cm</t>
+          <t>300-350 cm</t>
         </is>
       </c>
       <c r="F891" t="inlineStr">
         <is>
-          <t>12/ 14</t>
+          <t>8/10</t>
         </is>
       </c>
       <c r="G891" t="inlineStr">
         <is>
-          <t>£185.00</t>
+          <t>£115.00</t>
         </is>
       </c>
       <c r="H891" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I891" s="4" t="inlineStr"/>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>17488</t>
+          <t>17395</t>
         </is>
       </c>
       <c r="B892" t="inlineStr">
@@ -35218,33 +35226,29 @@
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>35Lt r</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E892" t="inlineStr">
         <is>
-          <t>400-450cm.cm</t>
-        </is>
-      </c>
-      <c r="F892" t="inlineStr">
-        <is>
-          <t>14/16</t>
-        </is>
-      </c>
+          <t>120-150cm</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr"/>
       <c r="G892" t="inlineStr">
         <is>
-          <t>£225.00</t>
+          <t>£24.00</t>
         </is>
       </c>
       <c r="H892" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I892" s="4" t="inlineStr"/>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
-          <t>17038</t>
+          <t>15652</t>
         </is>
       </c>
       <c r="B893" t="inlineStr">
@@ -35259,162 +35263,162 @@
       </c>
       <c r="D893" t="inlineStr">
         <is>
-          <t>35Ltr.</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E893" t="inlineStr">
         <is>
-          <t>350-400cm</t>
-        </is>
-      </c>
-      <c r="F893" t="inlineStr">
-        <is>
-          <t>10/ 12</t>
-        </is>
-      </c>
+          <t>200-250cm</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr"/>
       <c r="G893" t="inlineStr">
         <is>
-          <t>£155.00</t>
+          <t>£48.00</t>
         </is>
       </c>
       <c r="H893" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I893" s="4" t="inlineStr"/>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
         <is>
-          <t>16060</t>
+          <t>17039</t>
         </is>
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia 'Autumn Spire'</t>
+          <t>SORBUS aucuparia</t>
         </is>
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>Upright Mountain Ash</t>
+          <t>Rowan or Mountain Ash</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>35 Ltr</t>
         </is>
       </c>
       <c r="E894" t="inlineStr">
         <is>
-          <t>125-150cm</t>
-        </is>
-      </c>
-      <c r="F894" t="inlineStr"/>
+          <t>350-400 cm</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>12/ 14</t>
+        </is>
+      </c>
       <c r="G894" t="inlineStr">
         <is>
-          <t>£34.50</t>
+          <t>£185.00</t>
         </is>
       </c>
       <c r="H894" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I894" s="4" t="inlineStr"/>
     </row>
     <row r="895">
       <c r="A895" t="inlineStr">
         <is>
-          <t>17677</t>
+          <t>17488</t>
         </is>
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia 'Autumn Spire'</t>
+          <t>SORBUS aucuparia</t>
         </is>
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>Upright Mountain Ash</t>
+          <t>Rowan or Mountain Ash</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>B/ R</t>
+          <t>35Lt r</t>
         </is>
       </c>
       <c r="E895" t="inlineStr">
         <is>
-          <t>300-350cm</t>
+          <t>400-450cm.cm</t>
         </is>
       </c>
       <c r="F895" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>14/16</t>
         </is>
       </c>
       <c r="G895" t="inlineStr">
         <is>
-          <t>£130.00</t>
+          <t>£225.00</t>
         </is>
       </c>
       <c r="H895" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I895" s="4" t="inlineStr"/>
     </row>
     <row r="896">
       <c r="A896" t="inlineStr">
         <is>
-          <t>17676</t>
+          <t>17038</t>
         </is>
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia 'Autumn Spire'</t>
+          <t>SORBUS aucuparia</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>Upright Mountain Ash</t>
+          <t>Rowan or Mountain Ash</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>B/R</t>
+          <t>35Ltr.</t>
         </is>
       </c>
       <c r="E896" t="inlineStr">
         <is>
-          <t>250-300cm</t>
+          <t>350-400cm</t>
         </is>
       </c>
       <c r="F896" t="inlineStr">
         <is>
-          <t>8/10</t>
+          <t>10/ 12</t>
         </is>
       </c>
       <c r="G896" t="inlineStr">
         <is>
-          <t>£105.00</t>
+          <t>£155.00</t>
         </is>
       </c>
       <c r="H896" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I896" s="4" t="inlineStr"/>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
         <is>
-          <t>17231</t>
+          <t>16060</t>
         </is>
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia 'Fastigiata'</t>
+          <t>SORBUS aucuparia 'Autumn Spire'</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>Upright Rowan</t>
+          <t>Upright Mountain Ash</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
@@ -35434,181 +35438,185 @@
         </is>
       </c>
       <c r="H897" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I897" s="4" t="inlineStr"/>
     </row>
     <row r="898">
       <c r="A898" t="inlineStr">
         <is>
-          <t>12587</t>
+          <t>17677</t>
         </is>
       </c>
       <c r="B898" t="inlineStr">
         <is>
-          <t>SORBUS aucuparia 'Sheerwater Seedling'</t>
+          <t>SORBUS aucuparia 'Autumn Spire'</t>
         </is>
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Upright Mountain Ash</t>
         </is>
       </c>
       <c r="D898" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>B/ R</t>
         </is>
       </c>
       <c r="E898" t="inlineStr">
         <is>
-          <t>200-225cm</t>
-        </is>
-      </c>
-      <c r="F898" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G898" t="inlineStr">
         <is>
-          <t>£45.00</t>
+          <t>£130.00</t>
         </is>
       </c>
       <c r="H898" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I898" s="4" t="inlineStr"/>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
         <is>
-          <t>11881</t>
+          <t>17676</t>
         </is>
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>SORBUS commixta</t>
+          <t>SORBUS aucuparia 'Autumn Spire'</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>Japanese Rowan</t>
+          <t>Upright Mountain Ash</t>
         </is>
       </c>
       <c r="D899" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E899" t="inlineStr">
         <is>
-          <t>140-160cm</t>
-        </is>
-      </c>
-      <c r="F899" t="inlineStr"/>
+          <t>250-300cm</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G899" t="inlineStr">
         <is>
-          <t>£37.50</t>
+          <t>£105.00</t>
         </is>
       </c>
       <c r="H899" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I899" s="4" t="inlineStr"/>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
         <is>
-          <t>16496</t>
+          <t>17231</t>
         </is>
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>SORBUS hupehensis 'Pink Pagoda'</t>
+          <t>Sorbus aucuparia 'Fastigiata'</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>Mountain Ash</t>
+          <t>Upright Rowan</t>
         </is>
       </c>
       <c r="D900" t="inlineStr">
         <is>
-          <t>25Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>350-400cm</t>
-        </is>
-      </c>
-      <c r="F900" t="inlineStr">
-        <is>
-          <t>10/12</t>
-        </is>
-      </c>
+          <t>125-150cm</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr"/>
       <c r="G900" t="inlineStr">
         <is>
-          <t>£145.00</t>
+          <t>£34.50</t>
         </is>
       </c>
       <c r="H900" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I900" s="4" t="inlineStr"/>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
         <is>
-          <t>11708</t>
+          <t>12587</t>
         </is>
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>SORBUS intermedia</t>
+          <t>SORBUS aucuparia 'Sheerwater Seedling'</t>
         </is>
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>Swedish Whitebeam</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>150-200cm</t>
+          <t>200-225cm</t>
         </is>
       </c>
       <c r="F901" t="inlineStr"/>
       <c r="G901" t="inlineStr">
         <is>
-          <t>£37.50</t>
+          <t>£45.00</t>
         </is>
       </c>
       <c r="H901" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I901" s="4" t="inlineStr"/>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
         <is>
-          <t>16498</t>
+          <t>17683</t>
         </is>
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>SORBUS intermedia</t>
+          <t>SORBUS aucuparia 'Sheerwater Seedling'</t>
         </is>
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>Swedish Whitebeam</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>25Ltr</t>
+          <t>B/ R</t>
         </is>
       </c>
       <c r="E902" t="inlineStr">
@@ -35618,28 +35626,28 @@
       </c>
       <c r="F902" t="inlineStr">
         <is>
-          <t>8/10</t>
+          <t>10/12</t>
         </is>
       </c>
       <c r="G902" t="inlineStr">
         <is>
-          <t>£135.00</t>
+          <t>£130.00</t>
         </is>
       </c>
       <c r="H902" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I902" s="4" t="inlineStr"/>
     </row>
     <row r="903">
       <c r="A903" t="inlineStr">
         <is>
-          <t>15704</t>
+          <t>17682</t>
         </is>
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>SORBUS pseudovilmorinii</t>
+          <t>SORBUS aucuparia 'Sheerwater Seedling'</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
@@ -35649,191 +35657,199 @@
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>B/R</t>
         </is>
       </c>
       <c r="E903" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F903" t="inlineStr"/>
+          <t>250-300cm</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G903" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£105.00</t>
         </is>
       </c>
       <c r="H903" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I903" s="4" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>11280</t>
+          <t>11881</t>
         </is>
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>SORBUS thur. 'Fastigiata'</t>
+          <t>SORBUS commixta</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>Hybrid Whitebeam, Service Tree</t>
+          <t>Japanese Rowan</t>
         </is>
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E904" t="inlineStr">
         <is>
-          <t>200-225cm</t>
+          <t>140-160cm</t>
         </is>
       </c>
       <c r="F904" t="inlineStr"/>
       <c r="G904" t="inlineStr">
         <is>
-          <t>£55.00</t>
+          <t>£37.50</t>
         </is>
       </c>
       <c r="H904" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I904" s="4" t="inlineStr"/>
     </row>
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>17217</t>
+          <t>16496</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
         <is>
-          <t>SORBUS torminalis</t>
+          <t>SORBUS hupehensis 'Pink Pagoda'</t>
         </is>
       </c>
       <c r="C905" t="inlineStr">
         <is>
-          <t>Wild Service Tree</t>
+          <t>Mountain Ash</t>
         </is>
       </c>
       <c r="D905" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>25Ltr</t>
         </is>
       </c>
       <c r="E905" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F905" t="inlineStr"/>
+          <t>350-400cm</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G905" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£145.00</t>
         </is>
       </c>
       <c r="H905" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="I905" s="4" t="inlineStr"/>
     </row>
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>11046</t>
+          <t>11708</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
         <is>
-          <t>SORBUS vilmorinii</t>
+          <t>SORBUS intermedia</t>
         </is>
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>Vilmorin's rowan</t>
+          <t>Swedish Whitebeam</t>
         </is>
       </c>
       <c r="D906" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E906" t="inlineStr">
         <is>
-          <t>300-350cm</t>
-        </is>
-      </c>
-      <c r="F906" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>150-200cm</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr"/>
       <c r="G906" t="inlineStr">
         <is>
-          <t>£95.00</t>
+          <t>£37.50</t>
         </is>
       </c>
       <c r="H906" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I906" s="4" t="inlineStr"/>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">
         <is>
-          <t>11282</t>
+          <t>16498</t>
         </is>
       </c>
       <c r="B907" t="inlineStr">
         <is>
-          <t>STEWARTIA pseudocamellia</t>
+          <t>SORBUS intermedia</t>
         </is>
       </c>
       <c r="C907" t="inlineStr">
         <is>
-          <t>Japanese Stewartia</t>
+          <t>Swedish Whitebeam</t>
         </is>
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>25Ltr</t>
         </is>
       </c>
       <c r="E907" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F907" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G907" t="inlineStr">
         <is>
-          <t>£34.50</t>
+          <t>£135.00</t>
         </is>
       </c>
       <c r="H907" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I907" s="4" t="inlineStr"/>
     </row>
     <row r="908">
       <c r="A908" t="inlineStr">
         <is>
-          <t>17493</t>
+          <t>15704</t>
         </is>
       </c>
       <c r="B908" t="inlineStr">
         <is>
-          <t>STYRAX japonicus</t>
+          <t>SORBUS pseudovilmorinii</t>
         </is>
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>Japanese Snowball</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="D908" t="inlineStr">
@@ -35843,71 +35859,71 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>100-125cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F908" t="inlineStr"/>
       <c r="G908" t="inlineStr">
         <is>
-          <t>£37.50</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H908" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="I908" s="4" t="inlineStr"/>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
         <is>
-          <t>11156</t>
+          <t>11280</t>
         </is>
       </c>
       <c r="B909" t="inlineStr">
         <is>
-          <t>SYRINGA vulgaris 'Madame Lemoine'</t>
+          <t>SORBUS thur. 'Fastigiata'</t>
         </is>
       </c>
       <c r="C909" t="inlineStr">
         <is>
-          <t>Lilac</t>
+          <t>Hybrid Whitebeam, Service Tree</t>
         </is>
       </c>
       <c r="D909" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>75-100cm</t>
+          <t>200-225cm</t>
         </is>
       </c>
       <c r="F909" t="inlineStr"/>
       <c r="G909" t="inlineStr">
         <is>
-          <t>£31.50</t>
+          <t>£55.00</t>
         </is>
       </c>
       <c r="H909" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I909" s="4" t="inlineStr"/>
     </row>
     <row r="910">
       <c r="A910" t="inlineStr">
         <is>
-          <t>1143</t>
+          <t>17217</t>
         </is>
       </c>
       <c r="B910" t="inlineStr">
         <is>
-          <t>TAXODIUM distichum</t>
+          <t>SORBUS torminalis</t>
         </is>
       </c>
       <c r="C910" t="inlineStr">
         <is>
-          <t>Swamp Cypress</t>
+          <t>Wild Service Tree</t>
         </is>
       </c>
       <c r="D910" t="inlineStr">
@@ -35917,108 +35933,112 @@
       </c>
       <c r="E910" t="inlineStr">
         <is>
-          <t>100-125cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F910" t="inlineStr"/>
       <c r="G910" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H910" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="I910" s="4" t="inlineStr"/>
     </row>
     <row r="911">
       <c r="A911" t="inlineStr">
         <is>
-          <t>17460</t>
+          <t>11046</t>
         </is>
       </c>
       <c r="B911" t="inlineStr">
         <is>
-          <t>TAXODIUM distichum</t>
+          <t>SORBUS vilmorinii</t>
         </is>
       </c>
       <c r="C911" t="inlineStr">
         <is>
-          <t>Swamp Cypress</t>
+          <t>Vilmorin's rowan</t>
         </is>
       </c>
       <c r="D911" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E911" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F911" t="inlineStr"/>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G911" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£95.00</t>
         </is>
       </c>
       <c r="H911" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="I911" s="4" t="inlineStr"/>
     </row>
     <row r="912">
       <c r="A912" t="inlineStr">
         <is>
-          <t>16421</t>
+          <t>11282</t>
         </is>
       </c>
       <c r="B912" t="inlineStr">
         <is>
-          <t>TAXODIUM distichum</t>
+          <t>STEWARTIA pseudocamellia</t>
         </is>
       </c>
       <c r="C912" t="inlineStr">
         <is>
-          <t>Swamp Cypress</t>
+          <t>Japanese Stewartia</t>
         </is>
       </c>
       <c r="D912" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E912" t="inlineStr">
         <is>
-          <t>150-175cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F912" t="inlineStr"/>
       <c r="G912" t="inlineStr">
         <is>
-          <t>£48.00</t>
+          <t>£34.50</t>
         </is>
       </c>
       <c r="H912" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I912" s="4" t="inlineStr"/>
     </row>
     <row r="913">
       <c r="A913" t="inlineStr">
         <is>
-          <t>1592</t>
+          <t>17493</t>
         </is>
       </c>
       <c r="B913" t="inlineStr">
         <is>
-          <t>TAXUS baccata</t>
+          <t>STYRAX japonicus</t>
         </is>
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>Yew</t>
+          <t>Japanese Snowball</t>
         </is>
       </c>
       <c r="D913" t="inlineStr">
@@ -36028,71 +36048,71 @@
       </c>
       <c r="E913" t="inlineStr">
         <is>
-          <t>90-120cm</t>
+          <t>100-125cm</t>
         </is>
       </c>
       <c r="F913" t="inlineStr"/>
       <c r="G913" t="inlineStr">
         <is>
-          <t>£22.50</t>
+          <t>£37.50</t>
         </is>
       </c>
       <c r="H913" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I913" s="4" t="inlineStr"/>
     </row>
     <row r="914">
       <c r="A914" t="inlineStr">
         <is>
-          <t>16233</t>
+          <t>11156</t>
         </is>
       </c>
       <c r="B914" t="inlineStr">
         <is>
-          <t>TAXUS baccata</t>
+          <t>SYRINGA vulgaris 'Madame Lemoine'</t>
         </is>
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>Yew</t>
+          <t>Lilac</t>
         </is>
       </c>
       <c r="D914" t="inlineStr">
         <is>
-          <t>7.5Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E914" t="inlineStr">
         <is>
-          <t>100-125cm</t>
+          <t>75-100cm</t>
         </is>
       </c>
       <c r="F914" t="inlineStr"/>
       <c r="G914" t="inlineStr">
         <is>
-          <t>£45.00</t>
+          <t>£31.50</t>
         </is>
       </c>
       <c r="H914" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I914" s="4" t="inlineStr"/>
     </row>
     <row r="915">
       <c r="A915" t="inlineStr">
         <is>
-          <t>16062</t>
+          <t>1143</t>
         </is>
       </c>
       <c r="B915" t="inlineStr">
         <is>
-          <t>TAXUS baccata 'Fastigiata Robusta'</t>
+          <t>TAXODIUM distichum</t>
         </is>
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>English Yew</t>
+          <t>Swamp Cypress</t>
         </is>
       </c>
       <c r="D915" t="inlineStr">
@@ -36102,219 +36122,219 @@
       </c>
       <c r="E915" t="inlineStr">
         <is>
-          <t>60-80cm</t>
+          <t>100-125cm</t>
         </is>
       </c>
       <c r="F915" t="inlineStr"/>
       <c r="G915" t="inlineStr">
         <is>
-          <t>£22.50</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H915" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="I915" s="4" t="inlineStr"/>
     </row>
     <row r="916">
       <c r="A916" t="inlineStr">
         <is>
-          <t>1144</t>
+          <t>17460</t>
         </is>
       </c>
       <c r="B916" t="inlineStr">
         <is>
-          <t>TAXUS baccata Fastigiata Aurea</t>
+          <t>TAXODIUM distichum</t>
         </is>
       </c>
       <c r="C916" t="inlineStr">
         <is>
-          <t>Golden Irish Yew</t>
+          <t>Swamp Cypress</t>
         </is>
       </c>
       <c r="D916" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E916" t="inlineStr">
         <is>
-          <t>50-75cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F916" t="inlineStr"/>
       <c r="G916" t="inlineStr">
         <is>
-          <t>£24.00</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H916" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I916" s="4" t="inlineStr"/>
     </row>
     <row r="917">
       <c r="A917" t="inlineStr">
         <is>
-          <t>1145</t>
+          <t>16421</t>
         </is>
       </c>
       <c r="B917" t="inlineStr">
         <is>
-          <t>TETRADIUM daniellii</t>
+          <t>TAXODIUM distichum</t>
         </is>
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>Bee-bee Tree</t>
+          <t>Swamp Cypress</t>
         </is>
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E917" t="inlineStr">
         <is>
-          <t>90-120cm</t>
+          <t>150-175cm</t>
         </is>
       </c>
       <c r="F917" t="inlineStr"/>
       <c r="G917" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£48.00</t>
         </is>
       </c>
       <c r="H917" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I917" s="4" t="inlineStr"/>
     </row>
     <row r="918">
       <c r="A918" t="inlineStr">
         <is>
-          <t>16323</t>
+          <t>1592</t>
         </is>
       </c>
       <c r="B918" t="inlineStr">
         <is>
-          <t>TETRADIUM daniellii</t>
+          <t>TAXUS baccata</t>
         </is>
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>Bee-bee Tree</t>
+          <t>Yew</t>
         </is>
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E918" t="inlineStr">
         <is>
-          <t>200-250cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F918" t="inlineStr"/>
       <c r="G918" t="inlineStr">
         <is>
-          <t>£65.00</t>
+          <t>£22.50</t>
         </is>
       </c>
       <c r="H918" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="I918" s="4" t="inlineStr"/>
     </row>
     <row r="919">
       <c r="A919" t="inlineStr">
         <is>
-          <t>16298</t>
+          <t>16233</t>
         </is>
       </c>
       <c r="B919" t="inlineStr">
         <is>
-          <t>THUJA occidentalis 'Smaragd'</t>
+          <t>TAXUS baccata</t>
         </is>
       </c>
       <c r="C919" t="inlineStr">
         <is>
-          <t>White Cedar</t>
+          <t>Yew</t>
         </is>
       </c>
       <c r="D919" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>7.5Ltr</t>
         </is>
       </c>
       <c r="E919" t="inlineStr">
         <is>
-          <t>90-120cm</t>
+          <t>100-125cm</t>
         </is>
       </c>
       <c r="F919" t="inlineStr"/>
       <c r="G919" t="inlineStr">
         <is>
-          <t>£22.50</t>
+          <t>£45.00</t>
         </is>
       </c>
       <c r="H919" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I919" s="4" t="inlineStr"/>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
         <is>
-          <t>12603</t>
+          <t>16062</t>
         </is>
       </c>
       <c r="B920" t="inlineStr">
         <is>
-          <t>THUJA occidentalis 'Smaragd'</t>
+          <t>TAXUS baccata 'Fastigiata Robusta'</t>
         </is>
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>White Cedar</t>
+          <t>English Yew</t>
         </is>
       </c>
       <c r="D920" t="inlineStr">
         <is>
-          <t>180Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E920" t="inlineStr">
         <is>
-          <t>300-325cm</t>
+          <t>60-80cm</t>
         </is>
       </c>
       <c r="F920" t="inlineStr"/>
       <c r="G920" t="inlineStr">
         <is>
-          <t>£280.00</t>
+          <t>£22.50</t>
         </is>
       </c>
       <c r="H920" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="I920" s="4" t="inlineStr"/>
     </row>
     <row r="921">
       <c r="A921" t="inlineStr">
         <is>
-          <t>16332</t>
+          <t>1144</t>
         </is>
       </c>
       <c r="B921" t="inlineStr">
         <is>
-          <t>THUJA plicata 'Atrovirens'</t>
+          <t>TAXUS baccata Fastigiata Aurea</t>
         </is>
       </c>
       <c r="C921" t="inlineStr">
         <is>
-          <t>Western Red Cedar</t>
+          <t>Golden Irish Yew</t>
         </is>
       </c>
       <c r="D921" t="inlineStr">
@@ -36324,34 +36344,34 @@
       </c>
       <c r="E921" t="inlineStr">
         <is>
-          <t>75-100cm</t>
+          <t>50-75cm</t>
         </is>
       </c>
       <c r="F921" t="inlineStr"/>
       <c r="G921" t="inlineStr">
         <is>
-          <t>£18.00</t>
+          <t>£24.00</t>
         </is>
       </c>
       <c r="H921" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="I921" s="4" t="inlineStr"/>
     </row>
     <row r="922">
       <c r="A922" t="inlineStr">
         <is>
-          <t>17464</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="B922" t="inlineStr">
         <is>
-          <t>THUJA plicata 'Gelderland'</t>
+          <t>TETRADIUM daniellii</t>
         </is>
       </c>
       <c r="C922" t="inlineStr">
         <is>
-          <t>Western Red Cedar</t>
+          <t>Bee-bee Tree</t>
         </is>
       </c>
       <c r="D922" t="inlineStr">
@@ -36361,300 +36381,292 @@
       </c>
       <c r="E922" t="inlineStr">
         <is>
-          <t>60-90cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F922" t="inlineStr"/>
       <c r="G922" t="inlineStr">
         <is>
-          <t>£18.00</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H922" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="I922" s="4" t="inlineStr"/>
     </row>
     <row r="923">
       <c r="A923" t="inlineStr">
         <is>
-          <t>16251</t>
+          <t>16323</t>
         </is>
       </c>
       <c r="B923" t="inlineStr">
         <is>
-          <t>THUJOPSIS dolabrata</t>
+          <t>TETRADIUM daniellii</t>
         </is>
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>Hiba Arborvitae</t>
+          <t>Bee-bee Tree</t>
         </is>
       </c>
       <c r="D923" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E923" t="inlineStr">
         <is>
-          <t>30-50cm</t>
+          <t>200-250cm</t>
         </is>
       </c>
       <c r="F923" t="inlineStr"/>
       <c r="G923" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£65.00</t>
         </is>
       </c>
       <c r="H923" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I923" s="4" t="inlineStr"/>
     </row>
     <row r="924">
       <c r="A924" t="inlineStr">
         <is>
-          <t>15742</t>
+          <t>16298</t>
         </is>
       </c>
       <c r="B924" t="inlineStr">
         <is>
-          <t>TILIA americana 'American Sentry'</t>
+          <t>THUJA occidentalis 'Smaragd'</t>
         </is>
       </c>
       <c r="C924" t="inlineStr">
         <is>
-          <t>Sentry Linden</t>
+          <t>White Cedar</t>
         </is>
       </c>
       <c r="D924" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E924" t="inlineStr">
         <is>
-          <t>450-500cm</t>
-        </is>
-      </c>
-      <c r="F924" t="inlineStr">
-        <is>
-          <t>12/14</t>
-        </is>
-      </c>
+          <t>90-120cm</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr"/>
       <c r="G924" t="inlineStr">
         <is>
-          <t>£185.00</t>
+          <t>£22.50</t>
         </is>
       </c>
       <c r="H924" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="I924" s="4" t="inlineStr"/>
     </row>
     <row r="925">
       <c r="A925" t="inlineStr">
         <is>
-          <t>11632</t>
+          <t>12603</t>
         </is>
       </c>
       <c r="B925" t="inlineStr">
         <is>
-          <t>TILIA cordata</t>
+          <t>THUJA occidentalis 'Smaragd'</t>
         </is>
       </c>
       <c r="C925" t="inlineStr">
         <is>
-          <t>Small-leaved Lime</t>
+          <t>White Cedar</t>
         </is>
       </c>
       <c r="D925" t="inlineStr">
         <is>
-          <t>3 Ltr</t>
+          <t>180Ltr</t>
         </is>
       </c>
       <c r="E925" t="inlineStr">
         <is>
-          <t>125-150 cm</t>
+          <t>300-325cm</t>
         </is>
       </c>
       <c r="F925" t="inlineStr"/>
       <c r="G925" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£280.00</t>
         </is>
       </c>
       <c r="H925" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="I925" s="4" t="inlineStr"/>
     </row>
     <row r="926">
       <c r="A926" t="inlineStr">
         <is>
-          <t>11634</t>
+          <t>16332</t>
         </is>
       </c>
       <c r="B926" t="inlineStr">
         <is>
-          <t>TILIA cordata</t>
+          <t>THUJA plicata 'Atrovirens'</t>
         </is>
       </c>
       <c r="C926" t="inlineStr">
         <is>
-          <t>Small-leaved Lime</t>
+          <t>Western Red Cedar</t>
         </is>
       </c>
       <c r="D926" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E926" t="inlineStr">
         <is>
-          <t>250-300cm</t>
-        </is>
-      </c>
-      <c r="F926" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>75-100cm</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr"/>
       <c r="G926" t="inlineStr">
         <is>
-          <t>£80.00</t>
+          <t>£18.00</t>
         </is>
       </c>
       <c r="H926" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I926" s="4" t="inlineStr"/>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
         <is>
-          <t>11526</t>
+          <t>17464</t>
         </is>
       </c>
       <c r="B927" t="inlineStr">
         <is>
-          <t>TILIA cordata</t>
+          <t>THUJA plicata 'Gelderland'</t>
         </is>
       </c>
       <c r="C927" t="inlineStr">
         <is>
-          <t>Small-leaved Lime</t>
+          <t>Western Red Cedar</t>
         </is>
       </c>
       <c r="D927" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E927" t="inlineStr">
         <is>
-          <t>400-450cm</t>
-        </is>
-      </c>
-      <c r="F927" t="inlineStr">
-        <is>
-          <t>14/16</t>
-        </is>
-      </c>
+          <t>60-90cm</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr"/>
       <c r="G927" t="inlineStr">
         <is>
-          <t>£215.00</t>
+          <t>£18.00</t>
         </is>
       </c>
       <c r="H927" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="I927" s="4" t="inlineStr"/>
     </row>
     <row r="928">
       <c r="A928" t="inlineStr">
         <is>
-          <t>17218</t>
+          <t>16251</t>
         </is>
       </c>
       <c r="B928" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Greenspire '</t>
+          <t>THUJOPSIS dolabrata</t>
         </is>
       </c>
       <c r="C928" t="inlineStr">
         <is>
-          <t>Small-Leaved Lime</t>
+          <t>Hiba Arborvitae</t>
         </is>
       </c>
       <c r="D928" t="inlineStr">
         <is>
-          <t>5 Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E928" t="inlineStr">
         <is>
-          <t>100-125cm</t>
+          <t>30-50cm</t>
         </is>
       </c>
       <c r="F928" t="inlineStr"/>
       <c r="G928" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H928" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I928" s="4" t="inlineStr"/>
     </row>
     <row r="929">
       <c r="A929" t="inlineStr">
         <is>
-          <t>16085</t>
+          <t>15742</t>
         </is>
       </c>
       <c r="B929" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Greenspire '</t>
+          <t>TILIA americana 'American Sentry'</t>
         </is>
       </c>
       <c r="C929" t="inlineStr">
         <is>
-          <t>Small-Leaved Lime</t>
+          <t>Sentry Linden</t>
         </is>
       </c>
       <c r="D929" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E929" t="inlineStr">
         <is>
-          <t>125-150cm</t>
-        </is>
-      </c>
-      <c r="F929" t="inlineStr"/>
+          <t>450-500cm</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>12/14</t>
+        </is>
+      </c>
       <c r="G929" t="inlineStr">
         <is>
-          <t>£37.50</t>
+          <t>£185.00</t>
         </is>
       </c>
       <c r="H929" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I929" s="4" t="inlineStr"/>
     </row>
     <row r="930">
       <c r="A930" t="inlineStr">
         <is>
-          <t>16270</t>
+          <t>11632</t>
         </is>
       </c>
       <c r="B930" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Winter Orange'</t>
+          <t>TILIA cordata</t>
         </is>
       </c>
       <c r="C930" t="inlineStr">
@@ -36664,34 +36676,34 @@
       </c>
       <c r="D930" t="inlineStr">
         <is>
-          <t>5 Ltr</t>
+          <t>3 Ltr</t>
         </is>
       </c>
       <c r="E930" t="inlineStr">
         <is>
-          <t>175-200cm</t>
+          <t>125-150 cm</t>
         </is>
       </c>
       <c r="F930" t="inlineStr"/>
       <c r="G930" t="inlineStr">
         <is>
-          <t>£34.50</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H930" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="I930" s="4" t="inlineStr"/>
     </row>
     <row r="931">
       <c r="A931" t="inlineStr">
         <is>
-          <t>17494</t>
+          <t>11634</t>
         </is>
       </c>
       <c r="B931" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Winter Orange'</t>
+          <t>TILIA cordata</t>
         </is>
       </c>
       <c r="C931" t="inlineStr">
@@ -36701,34 +36713,38 @@
       </c>
       <c r="D931" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E931" t="inlineStr">
         <is>
-          <t>100-125cm</t>
-        </is>
-      </c>
-      <c r="F931" t="inlineStr"/>
+          <t>250-300cm</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G931" t="inlineStr">
         <is>
-          <t>£31.50</t>
+          <t>£80.00</t>
         </is>
       </c>
       <c r="H931" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="I931" s="4" t="inlineStr"/>
     </row>
     <row r="932">
       <c r="A932" t="inlineStr">
         <is>
-          <t>17420</t>
+          <t>11526</t>
         </is>
       </c>
       <c r="B932" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Winter Orange'</t>
+          <t>TILIA cordata</t>
         </is>
       </c>
       <c r="C932" t="inlineStr">
@@ -36738,122 +36754,122 @@
       </c>
       <c r="D932" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E932" t="inlineStr">
         <is>
-          <t>200-250cm</t>
-        </is>
-      </c>
-      <c r="F932" t="inlineStr"/>
+          <t>400-450cm</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>14/16</t>
+        </is>
+      </c>
       <c r="G932" t="inlineStr">
         <is>
-          <t>£55.00</t>
+          <t>£215.00</t>
         </is>
       </c>
       <c r="H932" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I932" s="4" t="inlineStr"/>
     </row>
     <row r="933">
       <c r="A933" t="inlineStr">
         <is>
-          <t>10713</t>
+          <t>17218</t>
         </is>
       </c>
       <c r="B933" t="inlineStr">
         <is>
-          <t>TILIA cordata 'Winter Orange'</t>
+          <t>TILIA cordata 'Greenspire '</t>
         </is>
       </c>
       <c r="C933" t="inlineStr">
         <is>
-          <t>Small-leaved Lime</t>
+          <t>Small-Leaved Lime</t>
         </is>
       </c>
       <c r="D933" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>5 Ltr</t>
         </is>
       </c>
       <c r="E933" t="inlineStr">
         <is>
-          <t>400-450cm</t>
-        </is>
-      </c>
-      <c r="F933" t="inlineStr">
-        <is>
-          <t>16/18</t>
-        </is>
-      </c>
+          <t>100-125cm</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr"/>
       <c r="G933" t="inlineStr">
         <is>
-          <t>£295.00</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H933" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="I933" s="4" t="inlineStr"/>
     </row>
     <row r="934">
       <c r="A934" t="inlineStr">
         <is>
-          <t>12405</t>
+          <t>16085</t>
         </is>
       </c>
       <c r="B934" t="inlineStr">
         <is>
-          <t>TILIA henryana</t>
+          <t>TILIA cordata 'Greenspire '</t>
         </is>
       </c>
       <c r="C934" t="inlineStr">
         <is>
-          <t>Henry's Lime</t>
+          <t>Small-Leaved Lime</t>
         </is>
       </c>
       <c r="D934" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E934" t="inlineStr">
         <is>
-          <t>90-120cm</t>
+          <t>125-150cm</t>
         </is>
       </c>
       <c r="F934" t="inlineStr"/>
       <c r="G934" t="inlineStr">
         <is>
-          <t>£31.50</t>
+          <t>£37.50</t>
         </is>
       </c>
       <c r="H934" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I934" s="4" t="inlineStr"/>
     </row>
     <row r="935">
       <c r="A935" t="inlineStr">
         <is>
-          <t>1603</t>
+          <t>16270</t>
         </is>
       </c>
       <c r="B935" t="inlineStr">
         <is>
-          <t>TILIA henryana</t>
+          <t>TILIA cordata 'Winter Orange'</t>
         </is>
       </c>
       <c r="C935" t="inlineStr">
         <is>
-          <t>Henry's Lime</t>
+          <t>Small-leaved Lime</t>
         </is>
       </c>
       <c r="D935" t="inlineStr">
         <is>
-          <t>20Ltr</t>
+          <t>5 Ltr</t>
         </is>
       </c>
       <c r="E935" t="inlineStr">
@@ -36861,72 +36877,68 @@
           <t>175-200cm</t>
         </is>
       </c>
-      <c r="F935" t="inlineStr">
-        <is>
-          <t>6/8</t>
-        </is>
-      </c>
+      <c r="F935" t="inlineStr"/>
       <c r="G935" t="inlineStr">
         <is>
-          <t>£85.00</t>
+          <t>£34.50</t>
         </is>
       </c>
       <c r="H935" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I935" s="4" t="inlineStr"/>
     </row>
     <row r="936">
       <c r="A936" t="inlineStr">
         <is>
-          <t>16287</t>
+          <t>17494</t>
         </is>
       </c>
       <c r="B936" t="inlineStr">
         <is>
-          <t>TILIA platyphyllos</t>
+          <t>TILIA cordata 'Winter Orange'</t>
         </is>
       </c>
       <c r="C936" t="inlineStr">
         <is>
-          <t>Broad-leaved Lime</t>
+          <t>Small-leaved Lime</t>
         </is>
       </c>
       <c r="D936" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E936" t="inlineStr">
         <is>
-          <t>120-150cm</t>
+          <t>100-125cm</t>
         </is>
       </c>
       <c r="F936" t="inlineStr"/>
       <c r="G936" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£31.50</t>
         </is>
       </c>
       <c r="H936" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="I936" s="4" t="inlineStr"/>
     </row>
     <row r="937">
       <c r="A937" t="inlineStr">
         <is>
-          <t>17449</t>
+          <t>17420</t>
         </is>
       </c>
       <c r="B937" t="inlineStr">
         <is>
-          <t>TILIA platyphyllos</t>
+          <t>TILIA cordata 'Winter Orange'</t>
         </is>
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>Broad-leaved Lime</t>
+          <t>Small-leaved Lime</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
@@ -36936,214 +36948,210 @@
       </c>
       <c r="E937" t="inlineStr">
         <is>
-          <t>250-300cm</t>
-        </is>
-      </c>
-      <c r="F937" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>200-250cm</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr"/>
       <c r="G937" t="inlineStr">
         <is>
-          <t>£75.00</t>
+          <t>£55.00</t>
         </is>
       </c>
       <c r="H937" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I937" s="4" t="inlineStr"/>
     </row>
     <row r="938">
       <c r="A938" t="inlineStr">
         <is>
-          <t>17421</t>
+          <t>10713</t>
         </is>
       </c>
       <c r="B938" t="inlineStr">
         <is>
-          <t>TILIA x euchlora</t>
+          <t>TILIA cordata 'Winter Orange'</t>
         </is>
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>European White Lime</t>
+          <t>Small-leaved Lime</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E938" t="inlineStr">
         <is>
-          <t>200-250cm</t>
-        </is>
-      </c>
-      <c r="F938" t="inlineStr"/>
+          <t>400-450cm</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>16/18</t>
+        </is>
+      </c>
       <c r="G938" t="inlineStr">
         <is>
-          <t>£55.00</t>
+          <t>£295.00</t>
         </is>
       </c>
       <c r="H938" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I938" s="4" t="inlineStr"/>
     </row>
     <row r="939">
       <c r="A939" t="inlineStr">
         <is>
-          <t>17220</t>
+          <t>12405</t>
         </is>
       </c>
       <c r="B939" t="inlineStr">
         <is>
-          <t>TILIA x europaea 'Pallida'</t>
+          <t>TILIA henryana</t>
         </is>
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>Kaiser Linden</t>
+          <t>Henry's Lime</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>5 Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E939" t="inlineStr">
         <is>
-          <t>120-150cm</t>
+          <t>90-120cm</t>
         </is>
       </c>
       <c r="F939" t="inlineStr"/>
       <c r="G939" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£31.50</t>
         </is>
       </c>
       <c r="H939" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I939" s="4" t="inlineStr"/>
     </row>
     <row r="940">
       <c r="A940" t="inlineStr">
         <is>
-          <t>16284</t>
+          <t>1603</t>
         </is>
       </c>
       <c r="B940" t="inlineStr">
         <is>
-          <t>TILIA x europaea 'Pallida'</t>
+          <t>TILIA henryana</t>
         </is>
       </c>
       <c r="C940" t="inlineStr">
         <is>
-          <t>Kaiser Linden</t>
+          <t>Henry's Lime</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>20Ltr</t>
         </is>
       </c>
       <c r="E940" t="inlineStr">
         <is>
-          <t>400-450cm</t>
+          <t>175-200cm</t>
         </is>
       </c>
       <c r="F940" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>6/8</t>
         </is>
       </c>
       <c r="G940" t="inlineStr">
         <is>
-          <t>£185.00</t>
+          <t>£85.00</t>
         </is>
       </c>
       <c r="H940" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I940" s="4" t="inlineStr"/>
     </row>
     <row r="941">
       <c r="A941" t="inlineStr">
         <is>
-          <t>11008</t>
+          <t>16287</t>
         </is>
       </c>
       <c r="B941" t="inlineStr">
         <is>
-          <t>TILIA x europaea 'Pallida'</t>
+          <t>TILIA platyphyllos</t>
         </is>
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>Kaiser Linden [5/yr pleached]</t>
+          <t>Broad-leaved Lime</t>
         </is>
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>230Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E941" t="inlineStr">
         <is>
-          <t>1.8x2x2mcm</t>
-        </is>
-      </c>
-      <c r="F941" t="inlineStr">
-        <is>
-          <t>25/30</t>
-        </is>
-      </c>
+          <t>120-150cm</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr"/>
       <c r="G941" t="inlineStr">
         <is>
-          <t>£650.00</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H941" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="I941" s="4" t="inlineStr"/>
     </row>
     <row r="942">
       <c r="A942" t="inlineStr">
         <is>
-          <t>13994</t>
+          <t>17449</t>
         </is>
       </c>
       <c r="B942" t="inlineStr">
         <is>
-          <t>TILIA x mongolica 'Harvest Gold'</t>
+          <t>TILIA platyphyllos</t>
         </is>
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>Mongolian Lime</t>
+          <t>Broad-leaved Lime</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>35 Ltr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E942" t="inlineStr">
         <is>
-          <t>250cm</t>
+          <t>250-300cm</t>
         </is>
       </c>
       <c r="F942" t="inlineStr">
         <is>
-          <t>6/8</t>
+          <t>8/10</t>
         </is>
       </c>
       <c r="G942" t="inlineStr">
         <is>
-          <t>£110.00</t>
+          <t>£75.00</t>
         </is>
       </c>
       <c r="H942" t="n">
@@ -37154,99 +37162,91 @@
     <row r="943">
       <c r="A943" t="inlineStr">
         <is>
-          <t>13995</t>
+          <t>17421</t>
         </is>
       </c>
       <c r="B943" t="inlineStr">
         <is>
-          <t>TILIA x mongolica 'Harvest Gold'</t>
+          <t>TILIA x euchlora</t>
         </is>
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>Mongolian Lime</t>
+          <t>European White Lime</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>35L tr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E943" t="inlineStr">
         <is>
-          <t>400-500cm</t>
-        </is>
-      </c>
-      <c r="F943" t="inlineStr">
-        <is>
-          <t>14/16</t>
-        </is>
-      </c>
+          <t>200-250cm</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr"/>
       <c r="G943" t="inlineStr">
         <is>
-          <t>£225.00</t>
+          <t>£55.00</t>
         </is>
       </c>
       <c r="H943" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I943" s="4" t="inlineStr"/>
     </row>
     <row r="944">
       <c r="A944" t="inlineStr">
         <is>
-          <t>17487</t>
+          <t>17220</t>
         </is>
       </c>
       <c r="B944" t="inlineStr">
         <is>
-          <t>TILIA x mongolica 'Harvest Gold'</t>
+          <t>TILIA x europaea 'Pallida'</t>
         </is>
       </c>
       <c r="C944" t="inlineStr">
         <is>
-          <t>Mongolian Lime</t>
+          <t>Kaiser Linden</t>
         </is>
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>35Lt r</t>
+          <t>5 Ltr</t>
         </is>
       </c>
       <c r="E944" t="inlineStr">
         <is>
-          <t>400-500 cm</t>
-        </is>
-      </c>
-      <c r="F944" t="inlineStr">
-        <is>
-          <t>16/18</t>
-        </is>
-      </c>
+          <t>120-150cm</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr"/>
       <c r="G944" t="inlineStr">
         <is>
-          <t>£260.00</t>
+          <t>£28.50</t>
         </is>
       </c>
       <c r="H944" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I944" s="4" t="inlineStr"/>
     </row>
     <row r="945">
       <c r="A945" t="inlineStr">
         <is>
-          <t>11169</t>
+          <t>16284</t>
         </is>
       </c>
       <c r="B945" t="inlineStr">
         <is>
-          <t>TILIA x mongolica 'Harvest Gold'</t>
+          <t>TILIA x europaea 'Pallida'</t>
         </is>
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>Mongolian Lime</t>
+          <t>Kaiser Linden</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
@@ -37261,273 +37261,289 @@
       </c>
       <c r="F945" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>12/14</t>
         </is>
       </c>
       <c r="G945" t="inlineStr">
         <is>
-          <t>£165.00</t>
+          <t>£185.00</t>
         </is>
       </c>
       <c r="H945" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I945" s="4" t="inlineStr"/>
     </row>
     <row r="946">
       <c r="A946" t="inlineStr">
         <is>
-          <t>17489</t>
+          <t>11008</t>
         </is>
       </c>
       <c r="B946" t="inlineStr">
         <is>
-          <t>TOONA sinensis</t>
+          <t>TILIA x europaea 'Pallida'</t>
         </is>
       </c>
       <c r="C946" t="inlineStr">
         <is>
-          <t>Chinese Cedar</t>
+          <t>Kaiser Linden [5/yr pleached]</t>
         </is>
       </c>
       <c r="D946" t="inlineStr">
         <is>
-          <t>35 Ltr</t>
+          <t>230Ltr</t>
         </is>
       </c>
       <c r="E946" t="inlineStr">
         <is>
-          <t>300-350cm.cm</t>
+          <t>1.8x2x2mcm</t>
         </is>
       </c>
       <c r="F946" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>25/30</t>
         </is>
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>£160.00</t>
+          <t>£650.00</t>
         </is>
       </c>
       <c r="H946" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I946" s="4" t="inlineStr"/>
     </row>
     <row r="947">
       <c r="A947" t="inlineStr">
         <is>
-          <t>10895</t>
+          <t>13994</t>
         </is>
       </c>
       <c r="B947" t="inlineStr">
         <is>
-          <t>TOONA sinensis</t>
+          <t>TILIA x mongolica 'Harvest Gold'</t>
         </is>
       </c>
       <c r="C947" t="inlineStr">
         <is>
-          <t>Chinese Cedar</t>
+          <t>Mongolian Lime</t>
         </is>
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>35Ltr</t>
+          <t>35 Ltr</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
         <is>
-          <t>300-350cm</t>
+          <t>250cm</t>
         </is>
       </c>
       <c r="F947" t="inlineStr">
         <is>
-          <t>8/10</t>
+          <t>6/8</t>
         </is>
       </c>
       <c r="G947" t="inlineStr">
         <is>
-          <t>£140.00</t>
+          <t>£110.00</t>
         </is>
       </c>
       <c r="H947" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I947" s="4" t="inlineStr"/>
     </row>
     <row r="948">
       <c r="A948" t="inlineStr">
         <is>
-          <t>16331</t>
+          <t>13995</t>
         </is>
       </c>
       <c r="B948" t="inlineStr">
         <is>
-          <t>TSUGA canadensis</t>
+          <t>TILIA x mongolica 'Harvest Gold'</t>
         </is>
       </c>
       <c r="C948" t="inlineStr">
         <is>
-          <t>Eastern Hemlock</t>
+          <t>Mongolian Lime</t>
         </is>
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>35L tr</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
         <is>
-          <t>75-100cm</t>
-        </is>
-      </c>
-      <c r="F948" t="inlineStr"/>
+          <t>400-500cm</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>14/16</t>
+        </is>
+      </c>
       <c r="G948" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£225.00</t>
         </is>
       </c>
       <c r="H948" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I948" s="4" t="inlineStr"/>
     </row>
     <row r="949">
       <c r="A949" t="inlineStr">
         <is>
-          <t>11779</t>
+          <t>17487</t>
         </is>
       </c>
       <c r="B949" t="inlineStr">
         <is>
-          <t>TSUGA canadensis</t>
+          <t>TILIA x mongolica 'Harvest Gold'</t>
         </is>
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>Eastern Hemlock</t>
+          <t>Mongolian Lime</t>
         </is>
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>12Ltr</t>
+          <t>35Lt r</t>
         </is>
       </c>
       <c r="E949" t="inlineStr">
         <is>
-          <t>140-160cm</t>
-        </is>
-      </c>
-      <c r="F949" t="inlineStr"/>
+          <t>400-500 cm</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>16/18</t>
+        </is>
+      </c>
       <c r="G949" t="inlineStr">
         <is>
-          <t>£60.00</t>
+          <t>£260.00</t>
         </is>
       </c>
       <c r="H949" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I949" s="4" t="inlineStr"/>
     </row>
     <row r="950">
       <c r="A950" t="inlineStr">
         <is>
-          <t>16318</t>
+          <t>11169</t>
         </is>
       </c>
       <c r="B950" t="inlineStr">
         <is>
-          <t>TSUGA heterophylla</t>
+          <t>TILIA x mongolica 'Harvest Gold'</t>
         </is>
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>Western Hemlock</t>
+          <t>Mongolian Lime</t>
         </is>
       </c>
       <c r="D950" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E950" t="inlineStr">
         <is>
-          <t>60-90cm</t>
-        </is>
-      </c>
-      <c r="F950" t="inlineStr"/>
+          <t>400-450cm</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G950" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£165.00</t>
         </is>
       </c>
       <c r="H950" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="I950" s="4" t="inlineStr"/>
     </row>
     <row r="951">
       <c r="A951" t="inlineStr">
         <is>
-          <t>14423</t>
+          <t>17489</t>
         </is>
       </c>
       <c r="B951" t="inlineStr">
         <is>
-          <t>ULMUS 'Lutece'</t>
+          <t>TOONA sinensis</t>
         </is>
       </c>
       <c r="C951" t="inlineStr">
         <is>
-          <t>Naguen Elm</t>
+          <t>Chinese Cedar</t>
         </is>
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>5Ltr</t>
+          <t>35 Ltr</t>
         </is>
       </c>
       <c r="E951" t="inlineStr">
         <is>
-          <t>100-125cm</t>
-        </is>
-      </c>
-      <c r="F951" t="inlineStr"/>
+          <t>300-350cm.cm</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
       <c r="G951" t="inlineStr">
         <is>
-          <t>£31.50</t>
+          <t>£160.00</t>
         </is>
       </c>
       <c r="H951" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I951" s="4" t="inlineStr"/>
     </row>
     <row r="952">
       <c r="A952" t="inlineStr">
         <is>
-          <t>14424</t>
+          <t>10895</t>
         </is>
       </c>
       <c r="B952" t="inlineStr">
         <is>
-          <t>ULMUS 'Lutece'</t>
+          <t>TOONA sinensis</t>
         </is>
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>Naguen Elm</t>
+          <t>Chinese Cedar</t>
         </is>
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>25Ltr</t>
+          <t>35Ltr</t>
         </is>
       </c>
       <c r="E952" t="inlineStr">
         <is>
-          <t>350-400cm</t>
+          <t>300-350cm</t>
         </is>
       </c>
       <c r="F952" t="inlineStr">
@@ -37537,152 +37553,144 @@
       </c>
       <c r="G952" t="inlineStr">
         <is>
-          <t>£95.00</t>
+          <t>£140.00</t>
         </is>
       </c>
       <c r="H952" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I952" s="4" t="inlineStr"/>
     </row>
     <row r="953">
       <c r="A953" t="inlineStr">
         <is>
-          <t>11601</t>
+          <t>16331</t>
         </is>
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>ULMUS 'Sapporo Autumn Gold'</t>
+          <t>TSUGA canadensis</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
         <is>
-          <t>Elm</t>
+          <t>Eastern Hemlock</t>
         </is>
       </c>
       <c r="D953" t="inlineStr">
         <is>
-          <t>20 Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E953" t="inlineStr">
         <is>
-          <t>300-350cm</t>
-        </is>
-      </c>
-      <c r="F953" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>75-100cm</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr"/>
       <c r="G953" t="inlineStr">
         <is>
-          <t>£95.00</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H953" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="I953" s="4" t="inlineStr"/>
     </row>
     <row r="954">
       <c r="A954" t="inlineStr">
         <is>
-          <t>11034</t>
+          <t>11779</t>
         </is>
       </c>
       <c r="B954" t="inlineStr">
         <is>
-          <t>ULMUS glabra 'Camperdownii'</t>
+          <t>TSUGA canadensis</t>
         </is>
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>Camperdown Elm</t>
+          <t>Eastern Hemlock</t>
         </is>
       </c>
       <c r="D954" t="inlineStr">
         <is>
-          <t>210Ltr</t>
+          <t>12Ltr</t>
         </is>
       </c>
       <c r="E954" t="inlineStr">
         <is>
-          <t>250-300cm</t>
-        </is>
-      </c>
-      <c r="F954" t="inlineStr">
-        <is>
-          <t>30/35</t>
-        </is>
-      </c>
+          <t>140-160cm</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr"/>
       <c r="G954" t="inlineStr">
         <is>
-          <t>£650.00</t>
+          <t>£60.00</t>
         </is>
       </c>
       <c r="H954" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I954" s="4" t="inlineStr"/>
     </row>
     <row r="955">
       <c r="A955" t="inlineStr">
         <is>
-          <t>17361</t>
+          <t>16318</t>
         </is>
       </c>
       <c r="B955" t="inlineStr">
         <is>
-          <t>ULMUS hollandica ‘Wredei’</t>
+          <t>TSUGA heterophylla</t>
         </is>
       </c>
       <c r="C955" t="inlineStr">
         <is>
-          <t>Golden Elm</t>
+          <t>Western Hemlock</t>
         </is>
       </c>
       <c r="D955" t="inlineStr">
         <is>
-          <t>20Ltr</t>
+          <t>3Ltr</t>
         </is>
       </c>
       <c r="E955" t="inlineStr">
         <is>
-          <t>150-200cm</t>
+          <t>60-90cm</t>
         </is>
       </c>
       <c r="F955" t="inlineStr"/>
       <c r="G955" t="inlineStr">
         <is>
-          <t>£65.00</t>
+          <t>£25.50</t>
         </is>
       </c>
       <c r="H955" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I955" s="4" t="inlineStr"/>
     </row>
     <row r="956">
       <c r="A956" t="inlineStr">
         <is>
-          <t>11709</t>
+          <t>14423</t>
         </is>
       </c>
       <c r="B956" t="inlineStr">
         <is>
-          <t>ZELKOVA serrata</t>
+          <t>ULMUS 'Lutece'</t>
         </is>
       </c>
       <c r="C956" t="inlineStr">
         <is>
-          <t>Japanese Zelkova</t>
+          <t>Naguen Elm</t>
         </is>
       </c>
       <c r="D956" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>5Ltr</t>
         </is>
       </c>
       <c r="E956" t="inlineStr">
@@ -37693,91 +37701,288 @@
       <c r="F956" t="inlineStr"/>
       <c r="G956" t="inlineStr">
         <is>
-          <t>£25.50</t>
+          <t>£31.50</t>
         </is>
       </c>
       <c r="H956" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I956" s="4" t="inlineStr"/>
     </row>
     <row r="957">
       <c r="A957" t="inlineStr">
         <is>
-          <t>17377</t>
+          <t>14424</t>
         </is>
       </c>
       <c r="B957" t="inlineStr">
         <is>
-          <t>ZELKOVA serrata 'Green Vase'</t>
+          <t>ULMUS 'Lutece'</t>
         </is>
       </c>
       <c r="C957" t="inlineStr">
         <is>
-          <t>Japanese Zelkova</t>
+          <t>Naguen Elm</t>
         </is>
       </c>
       <c r="D957" t="inlineStr">
         <is>
-          <t>3Ltr</t>
+          <t>25Ltr</t>
         </is>
       </c>
       <c r="E957" t="inlineStr">
         <is>
-          <t>90-120cm</t>
-        </is>
-      </c>
-      <c r="F957" t="inlineStr"/>
+          <t>350-400cm</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
       <c r="G957" t="inlineStr">
         <is>
-          <t>£28.50</t>
+          <t>£95.00</t>
         </is>
       </c>
       <c r="H957" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="I957" s="4" t="inlineStr"/>
     </row>
     <row r="958">
       <c r="A958" t="inlineStr">
         <is>
+          <t>11601</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>ULMUS 'Sapporo Autumn Gold'</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Elm</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>20 Ltr</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>300-350cm</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>£95.00</t>
+        </is>
+      </c>
+      <c r="H958" t="n">
+        <v>3</v>
+      </c>
+      <c r="I958" s="4" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>11034</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>ULMUS glabra 'Camperdownii'</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Camperdown Elm</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>210Ltr</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>250-300cm</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>30/35</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>£650.00</t>
+        </is>
+      </c>
+      <c r="H959" t="n">
+        <v>2</v>
+      </c>
+      <c r="I959" s="4" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>17361</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>ULMUS hollandica ‘Wredei’</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Golden Elm</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>20Ltr</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>150-200cm</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr"/>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>£65.00</t>
+        </is>
+      </c>
+      <c r="H960" t="n">
+        <v>4</v>
+      </c>
+      <c r="I960" s="4" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>11709</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>ZELKOVA serrata</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Japanese Zelkova</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>3Ltr</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>100-125cm</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr"/>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>£25.50</t>
+        </is>
+      </c>
+      <c r="H961" t="n">
+        <v>12</v>
+      </c>
+      <c r="I961" s="4" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>17377</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>ZELKOVA serrata 'Green Vase'</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Japanese Zelkova</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>3Ltr</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>90-120cm</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr"/>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>£28.50</t>
+        </is>
+      </c>
+      <c r="H962" t="n">
+        <v>28</v>
+      </c>
+      <c r="I962" s="4" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
           <t>11168</t>
         </is>
       </c>
-      <c r="B958" t="inlineStr">
+      <c r="B963" t="inlineStr">
         <is>
           <t>ZELKOVA serrata 'Green Vase'</t>
         </is>
       </c>
-      <c r="C958" t="inlineStr">
+      <c r="C963" t="inlineStr">
         <is>
           <t>Japanese Zelkova</t>
         </is>
       </c>
-      <c r="D958" t="inlineStr">
+      <c r="D963" t="inlineStr">
         <is>
           <t>25Ltr</t>
         </is>
       </c>
-      <c r="E958" t="inlineStr">
+      <c r="E963" t="inlineStr">
         <is>
           <t>250-300cm</t>
         </is>
       </c>
-      <c r="F958" t="inlineStr">
+      <c r="F963" t="inlineStr">
         <is>
           <t>6/8</t>
         </is>
       </c>
-      <c r="G958" t="inlineStr">
+      <c r="G963" t="inlineStr">
         <is>
           <t>£95.00</t>
         </is>
       </c>
-      <c r="H958" t="n">
+      <c r="H963" t="n">
         <v>4</v>
       </c>
-      <c r="I958" s="4" t="inlineStr"/>
+      <c r="I963" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>